<commit_message>
Index-first universe, live spread sizing, intraday/VIX/IC regime tests (Stages 8g-8m)
- ADX>20 entry filter for stocks; rising-ADX variant tested and rejected
- Intraday setups tested on 5-min data: nothing survives costs (8h)
- Indices vs NIFTY 50 vs other stocks (8i); VIX regime test (8j)
- spread_builder: live strikes, credit, Kite margin, lots by max loss (8k)
- Strike distance model (8l); NIFTY IC vs credit spread regime rule rejected (8m)
- Journal records spread and sizing fields; SENSEX via BSE/BFO

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/ADANIPORTS_full_report.xlsx
+++ b/exports/ADANIPORTS_full_report.xlsx
@@ -4375,7 +4375,7 @@
         <v>0</v>
       </c>
       <c r="Q69" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -6398,16 +6398,16 @@
         <v>1674.2</v>
       </c>
       <c r="E59" t="n">
-        <v>1746.7</v>
+        <v>1755</v>
       </c>
       <c r="F59" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G59" t="n">
         <v>6.43</v>
       </c>
       <c r="H59" t="n">
-        <v>-2.2</v>
+        <v>-1.74</v>
       </c>
       <c r="I59" t="n">
         <v>0.17</v>

</xml_diff>